<commit_message>
Define Android pilot scope and feasibility budget
</commit_message>
<xml_diff>
--- a/ProofCam_Android_Development_Roadmap.xlsx
+++ b/ProofCam_Android_Development_Roadmap.xlsx
@@ -166,6 +166,11 @@
     <comment ref="J2" authorId="0" shapeId="0">
       <text>
         <t>Step 1 documented in docs/01-product-brief.md. Working product decisions established under the instruction to proceed; external validation and implementation remain pending.</t>
+      </text>
+    </comment>
+    <comment ref="J3" authorId="0" shapeId="0">
+      <text>
+        <t>Planning complete: docs/02-pilot-scope-and-budget.md. Android 14+, three reference configurations, ownership, scoped pilot, and $2,000 feasibility proposal. Actual spending authorization remains $0; purchases and device access are pending.</t>
       </text>
     </comment>
   </commentList>
@@ -633,7 +638,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Product + engineering leads</t>
+          <t>Armaan Singh (accountable); Codex (documentation)</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -643,7 +648,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Complete</t>
         </is>
       </c>
     </row>
@@ -1556,13 +1561,14 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1660,7 +1666,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Kotlin/Compose/CameraX and Rust shared integrity/backend are proposed working choices. Watermark runtime, cloud provider, minimum OS, devices, and exact protocol details are finalized at the indicated gates.</t>
+          <t>Android pilot floor: Android 14/API 34, arm64-v8a. Reference targets: Galaxy A15 5G 4/128 GB, Pixel 8a 8/128 GB, Galaxy S24 US 8/128 GB. Kotlin/Compose/CameraX and Rust remain working technology choices; watermark runtime and protocol details await later gates.</t>
         </is>
       </c>
     </row>
@@ -1696,7 +1702,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Suggested roles are placeholders, not assigned people. Budget and purchases require approval. No dates or duration commitments until the feasibility gate.</t>
+          <t>Armaan Singh is accountable; Codex assists with documentation and implementation when tasked. Independent security reviewer remains to be appointed. See docs/02-pilot-scope-and-budget.md. No purchase authorization or release date.</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1738,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Use the Status dropdown on the roadmap. All goals start as Not started. Completion criteria describe evidence required before marking Complete.</t>
+          <t>Use the Status dropdown. Goals 1 and 2 have completed planning documents; goals 3–20 remain Not started. Planning completion does not imply purchase authorization, physical validation, or implementation.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace feasibility budget with free-development constraint
</commit_message>
<xml_diff>
--- a/ProofCam_Android_Development_Roadmap.xlsx
+++ b/ProofCam_Android_Development_Roadmap.xlsx
@@ -170,7 +170,7 @@
     </comment>
     <comment ref="J3" authorId="0" shapeId="0">
       <text>
-        <t>Planning complete: docs/02-pilot-scope-and-budget.md. Android 14+, three reference configurations, ownership, scoped pilot, and $2,000 feasibility proposal. Actual spending authorization remains $0; purchases and device access are pending.</t>
+        <t>Planning complete; supersedes the paid feasibility proposal. Use existing/free resources only. Actual device inventory and measurements remain pending. See docs/02-pilot-scope-and-free-development.md.</t>
       </text>
     </comment>
   </commentList>
@@ -613,7 +613,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Freeze pilot scope and feasibility budget</t>
+          <t>Freeze pilot scope and free-development constraints</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -623,12 +623,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Scope, device shortlist, budget proposal, and deferred-feature list.</t>
+          <t>Scope, available-hardware plan, free-tooling constraints, and deferred-feature list.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Name three Android reference devices; assign owners and approve spending before purchases; defer iOS, video, editing, and browser UI.</t>
+          <t>Define Android support and reference tiers; assign accountability; use existing or freely borrowed devices and no paid services; defer iOS, video, editing, and browser UI.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -878,7 +878,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Fit 128-bit ID plus routing/coding or explicitly approve a capacity redesign; pass an initial three-device feasibility review before committing to release timing.</t>
+          <t>Fit 128-bit ID plus routing/coding or explicitly document a capacity redesign; complete feasibility on available physical devices, list untested tiers, and restrict support claims accordingly.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -1173,7 +1173,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Registration service, immutable database records, KMS signing, and idempotent retry handling.</t>
+          <t>Registration service, immutable records, protected server signing, and idempotent retries; development trust kept separate.</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Rust/Axum; PostgreSQL; managed KMS; CAP5–7; OPS1</t>
+          <t>Rust/Axum; PostgreSQL; free/local signing prototype; trusted public signing remains gated by CAP7 and SEC3.</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
@@ -1393,7 +1393,7 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>Proposed AWS ECS/RDS/S3/KMS; Terraform; SEC4–5; OPS1–5</t>
+          <t>Existing infrastructure or verified no-cost hosting; local prototype otherwise; SEC4–5; OPS1–5.</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
@@ -1478,7 +1478,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>At least 9/10 reviewers distinguish recovery from integrity; critical issues resolved; rerun affected checks; verify current store requirements before submission.</t>
+          <t>At least 9/10 reviewers distinguish recovery from integrity; critical issues resolved; rerun affected checks; document direct-APK distribution and available attestation evidence.</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1493,7 +1493,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Google Play closed testing; delivery step 6</t>
+          <t>Direct signed-APK closed pilot; delivery step 6</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1543,7 +1543,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Google Play staged rollout; production monitoring</t>
+          <t>Direct signed-APK staged rollout; no-cost hosting if compliant; production monitoring.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -1579,7 +1579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1666,7 +1666,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Android pilot floor: Android 14/API 34, arm64-v8a. Reference targets: Galaxy A15 5G 4/128 GB, Pixel 8a 8/128 GB, Galaxy S24 US 8/128 GB. Kotlin/Compose/CameraX and Rust remain working technology choices; watermark runtime and protocol details await later gates.</t>
+          <t>Android pilot floor: Android 14/API 34, arm64-v8a. Illustrative comparison targets, not required purchases: Galaxy A15 5G 4/128 GB, Pixel 8a 8/128 GB, Galaxy S24 US 8/128 GB. Kotlin/Compose/CameraX and Rust remain working technology choices; watermark runtime and protocol details await later gates.</t>
         </is>
       </c>
     </row>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Armaan Singh is accountable; Codex assists with documentation and implementation when tasked. Independent security reviewer remains to be appointed. See docs/02-pilot-scope-and-budget.md. No purchase authorization or release date.</t>
+          <t>Armaan Singh is accountable; Codex assists with documentation and implementation when tasked. Independent security reviewer remains to be appointed. See docs/02-pilot-scope-and-free-development.md. Free resources only; no release date.</t>
         </is>
       </c>
     </row>
@@ -1738,7 +1738,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Use the Status dropdown. Goals 1 and 2 have completed planning documents; goals 3–20 remain Not started. Planning completion does not imply purchase authorization, physical validation, or implementation.</t>
+          <t>Use the Status dropdown. Goals 1 and 2 have completed planning documents; goals 3–20 remain Not started. Planning completion does not imply physical validation or implementation.</t>
         </is>
       </c>
     </row>
@@ -1751,6 +1751,18 @@
       <c r="B14" s="3" t="inlineStr">
         <is>
           <t>Check then-current platform, SDK, attestation, and Google Play policies during implementation and before release. This workbook is not a current-policy audit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="75" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Free-development constraint</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Existing or freely borrowed devices; local compute; free tools and licensed data; no paid services or store enrollment. Direct signed APK distribution. Public hosting/signing remains gated on compliant no-cost resources; never claim unavailable attestation.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Define threat model privacy and capture assurance policy
</commit_message>
<xml_diff>
--- a/ProofCam_Android_Development_Roadmap.xlsx
+++ b/ProofCam_Android_Development_Roadmap.xlsx
@@ -171,6 +171,11 @@
     <comment ref="J3" authorId="0" shapeId="0">
       <text>
         <t>Planning complete; supersedes the paid feasibility proposal. Use existing/free resources only. Actual device inventory and measurements remain pending. See docs/02-pilot-scope-and-free-development.md.</t>
+      </text>
+    </comment>
+    <comment ref="J4" authorId="0" shapeId="0">
+      <text>
+        <t>Policy baseline complete: threat register T01–T14, assurance matrix, data map, retention/removal, and release gates. Implementation and independent review pending.</t>
       </text>
     </comment>
   </commentList>
@@ -688,7 +693,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Security + product leads</t>
+          <t>Armaan Singh (accountable); Codex (policy documentation)</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -698,7 +703,7 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Complete</t>
         </is>
       </c>
     </row>
@@ -1562,13 +1567,14 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1738,7 +1744,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Use the Status dropdown. Goals 1 and 2 have completed planning documents; goals 3–20 remain Not started. Planning completion does not imply physical validation or implementation.</t>
+          <t>Use the Status dropdown. Goals 1–3 have completed planning documents; goals 4–20 remain Not started. Policy completion does not mean implementation, physical validation, or security audit.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Design capture and verification flows with interactive prototype
</commit_message>
<xml_diff>
--- a/ProofCam_Android_Development_Roadmap.xlsx
+++ b/ProofCam_Android_Development_Roadmap.xlsx
@@ -176,6 +176,11 @@
     <comment ref="J4" authorId="0" shapeId="0">
       <text>
         <t>Policy baseline complete: threat register T01–T14, assurance matrix, data map, retention/removal, and release gates. Implementation and independent review pending.</t>
+      </text>
+    </comment>
+    <comment ref="J5" authorId="0" shapeId="0">
+      <text>
+        <t>Screen specification, lifecycle diagrams, failure-state copy, and local interactive prototype delivered. Syntax and 33 prototype logic assertions passed. Browser visual review, user testing, and Android implementation remain pending.</t>
       </text>
     </comment>
   </commentList>
@@ -743,7 +748,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Product designer</t>
+          <t>Armaan Singh (accountable); Codex (design/prototype)</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -753,7 +758,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Complete</t>
         </is>
       </c>
     </row>
@@ -1568,13 +1573,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1744,7 +1750,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Use the Status dropdown. Goals 1–3 have completed planning documents; goals 4–20 remain Not started. Policy completion does not mean implementation, physical validation, or security audit.</t>
+          <t>Goals 1–4 have completed planning/design artifacts; goals 5–20 remain Not started. The interactive prototype is simulated; implementation, native-device validation, and user review remain pending.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add photo benchmark harness and locked starter corpus
</commit_message>
<xml_diff>
--- a/ProofCam_Android_Development_Roadmap.xlsx
+++ b/ProofCam_Android_Development_Roadmap.xlsx
@@ -181,6 +181,11 @@
     <comment ref="J5" authorId="0" shapeId="0">
       <text>
         <t>Screen specification, lifecycle diagrams, failure-state copy, and local interactive prototype delivered. Syntax and 33 prototype logic assertions passed. Browser visual review, user testing, and Android implementation remain pending.</t>
+      </text>
+    </comment>
+    <comment ref="J6" authorId="0" shapeId="0">
+      <text>
+        <t>Harness and 1,200-source starter snapshot delivered: 100 tuning, 1,000 held-out, 100 negative candidates. Full 300,000-input negative suite, rights/category/near-duplicate review, and actual screenshot collection remain pending. See benchmark/reports and goal 5 readiness document.</t>
       </text>
     </comment>
   </commentList>
@@ -798,7 +803,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>QA + watermark engineers</t>
+          <t>Armaan Singh (accountable); Codex (harness/acquisition)</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -808,7 +813,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
     </row>
@@ -1574,13 +1579,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1750,7 +1756,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Goals 1–4 have completed planning/design artifacts; goals 5–20 remain Not started. The interactive prototype is simulated; implementation, native-device validation, and user review remain pending.</t>
+          <t>Goals 1–4 have completed planning/design artifacts. Goal 5 is In progress: harness and starter corpus delivered, release data readiness pending. Goals 6–20 remain Not started. Goal 6 may use tuning data while corpus work continues.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Expand benchmark corpus and add evidence readiness tooling
</commit_message>
<xml_diff>
--- a/ProofCam_Android_Development_Roadmap.xlsx
+++ b/ProofCam_Android_Development_Roadmap.xlsx
@@ -185,7 +185,7 @@
     </comment>
     <comment ref="J6" authorId="0" shapeId="0">
       <text>
-        <t>Harness and 1,200-source starter snapshot delivered: 100 tuning, 1,000 held-out, 100 negative candidates. Full 300,000-input negative suite, rights/category/near-duplicate review, and actual screenshot collection remain pending. See benchmark/reports and goal 5 readiness document.</t>
+        <t>Continued: 11,200 distinct source images (100 tuning / 1,000 held-out / 10,100 negative), 53 native-2048+ variants, 300,000 pinned stress recipes over 10,000 parents, paginated review and screenshot intake. 32 tests pass. Local approval, physical screenshots, and final negative input/statistical eligibility remain pending; recipes are not independent photographs or completed evaluations.</t>
       </text>
     </comment>
   </commentList>
@@ -1756,7 +1756,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Goals 1–4 have completed planning/design artifacts. Goal 5 is In progress: harness and starter corpus delivered, release data readiness pending. Goals 6–20 remain Not started. Goal 6 may use tuning data while corpus work continues.</t>
+          <t>Goals 1–4 planning/design complete. Goal 5 In progress: expanded corpus and data tooling delivered, with physical evidence and final review/eligibility pending. 300,000 stress recipes share 10,000 source parents. Goals 6–20 Not started; tuning experiments may proceed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record tuning corpus visual review with scoped validation
</commit_message>
<xml_diff>
--- a/ProofCam_Android_Development_Roadmap.xlsx
+++ b/ProofCam_Android_Development_Roadmap.xlsx
@@ -161,6 +161,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>ProofCam</author>
+    <author>Codex</author>
   </authors>
   <commentList>
     <comment ref="J2" authorId="0" shapeId="0">
@@ -183,9 +184,9 @@
         <t>Screen specification, lifecycle diagrams, failure-state copy, and local interactive prototype delivered. Syntax and 33 prototype logic assertions passed. Browser visual review, user testing, and Android implementation remain pending.</t>
       </text>
     </comment>
-    <comment ref="J6" authorId="0" shapeId="0">
+    <comment ref="J6" authorId="1" shapeId="0">
       <text>
-        <t>Continued: 11,200 distinct source images (100 tuning / 1,000 held-out / 10,100 negative), 53 native-2048+ variants, 300,000 pinned stress recipes over 10,000 parents, paginated review and screenshot intake. 32 tests pass. Local approval, physical screenshots, and final negative input/statistical eligibility remain pending; recipes are not independent photographs or completed evaluations.</t>
+        <t>100 tuning images visually screened by Codex; this is not rights or release approval. See benchmark/reviews/tuning-visual-v1.json. 34 automated tests pass.</t>
       </text>
     </comment>
   </commentList>
@@ -1756,7 +1757,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Goals 1–4 planning/design complete. Goal 5 In progress: expanded corpus and data tooling delivered, with physical evidence and final review/eligibility pending. 300,000 stress recipes share 10,000 source parents. Goals 6–20 Not started; tuning experiments may proceed.</t>
+          <t>Goals 1–4 planning/design complete. Goal 5 In progress: corpus/harness delivered; AI visual screening of 100 tuning images recommends 92 primary-photo candidates and 8 separate stress examples. Rights, held-out/negative review, and real screenshots pending. 300,000 stress recipes share 10,000 parents. Goals 6–20 Not started.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Start conventional watermark benchmarks with two measured DCT baselines
</commit_message>
<xml_diff>
--- a/ProofCam_Android_Development_Roadmap.xlsx
+++ b/ProofCam_Android_Development_Roadmap.xlsx
@@ -187,6 +187,11 @@
     <comment ref="J6" authorId="1" shapeId="0">
       <text>
         <t>100 tuning images visually screened by Codex; this is not rights or release approval. See benchmark/reviews/tuning-visual-v1.json. 34 automated tests pass.</t>
+      </text>
+    </comment>
+    <comment ref="J7" authorId="1" shapeId="0">
+      <text>
+        <t>Initial comparison completed: 1,592 desktop searches across two conventional DCT baselines, 24 tuning photos and 100 negative candidates. Neither meets quality or geometric recovery requirements. 37 tests pass. Goal remains In progress; actual screenshots, Android measurements, further candidates and final license review pending.</t>
       </text>
     </comment>
   </commentList>
@@ -854,7 +859,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Watermark engineer</t>
+          <t>Armaan Singh (accountable); Codex (research implementation)</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -864,7 +869,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
     </row>
@@ -1757,7 +1762,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Goals 1–4 planning/design complete. Goal 5 In progress: corpus/harness delivered; AI visual screening of 100 tuning images recommends 92 primary-photo candidates and 8 separate stress examples. Rights, held-out/negative review, and real screenshots pending. 300,000 stress recipes share 10,000 parents. Goals 6–20 Not started.</t>
+          <t>Goals 1–4 planning/design complete. Goal 5 In progress: rights, held-out/negative review, and actual screenshots pending. Goal 6 In progress: two conventional full-ID DCT baselines and initial desktop tuning comparison. Goals 7–20 Not started. No production watermark selected.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Improve conventional watermark quality and bounded scale recovery
</commit_message>
<xml_diff>
--- a/ProofCam_Android_Development_Roadmap.xlsx
+++ b/ProofCam_Android_Development_Roadmap.xlsx
@@ -191,7 +191,7 @@
     </comment>
     <comment ref="J7" authorId="1" shapeId="0">
       <text>
-        <t>Initial comparison completed: 1,592 desktop searches across two conventional DCT baselines, 24 tuning photos and 100 negative candidates. Neither meets quality or geometric recovery requirements. 37 tests pass. Goal remains In progress; actual screenshots, Android measurements, further candidates and final license review pending.</t>
+        <t>v2 completed 1,592 desktop cases. Gentler QIM meets the numerical quality floor on 24 tuning photos: mean SSIM 0.99127; 24/24 original and 1024 synthetic screenshot IDs, 21/24 at 512. Both candidates fail crop/rotation. 40 tests pass and sample replay matches. Real screenshots, Android cost and final candidate selection pending.</t>
       </text>
     </comment>
   </commentList>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Goals 1–4 planning/design complete. Goal 5 In progress: rights, held-out/negative review, and actual screenshots pending. Goal 6 In progress: two conventional full-ID DCT baselines and initial desktop tuning comparison. Goals 7–20 Not started. No production watermark selected.</t>
+          <t>Goals 1–4 planning/design complete. Goal 5 In progress: rights, held-out/negative review and real screenshots pending. Goal 6 In progress: conventional DCT baseline comparisons now include lower-strength embedding and bounded scale/border recovery. Goals 7–20 Not started; no production candidate selected.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Conclude desktop feasibility and prepare Android benchmark; record device blocker
</commit_message>
<xml_diff>
--- a/ProofCam_Android_Development_Roadmap.xlsx
+++ b/ProofCam_Android_Development_Roadmap.xlsx
@@ -191,7 +191,7 @@
     </comment>
     <comment ref="J7" authorId="1" shapeId="0">
       <text>
-        <t>v2 completed 1,592 desktop cases. Gentler QIM meets the numerical quality floor on 24 tuning photos: mean SSIM 0.99127; 24/24 original and 1024 synthetic screenshot IDs, 21/24 at 512. Both candidates fail crop/rotation. 40 tests pass and sample replay matches. Real screenshots, Android cost and final candidate selection pending.</t>
+        <t>Desktop study complete: 3,668 scheduled cases on 92 positive and 1,000 negative candidates, plus 45 native-resolution variant cases. One positive/six negative ICC failures retained. Android research APK built and host core tests pass. User confirmed no phone on 2026-09-26. Actual screenshots, native latency/peak memory and display artifact checks are unmeasured; no production candidate selected.</t>
       </text>
     </comment>
   </commentList>
@@ -869,7 +869,7 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Blocked — device unavailable</t>
         </is>
       </c>
     </row>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Goals 1–4 planning/design complete. Goal 5 In progress: rights, held-out/negative review and real screenshots pending. Goal 6 In progress: conventional DCT baseline comparisons now include lower-strength embedding and bounded scale/border recovery. Goals 7–20 Not started; no production candidate selected.</t>
+          <t>Goals 1–4 planning/design complete. Goal 5 In progress (rights/final corpus/device evidence). Goal 6 desktop work complete; full goal Blocked — device unavailable, confirmed 2026-09-26. Research Android APK built; physical tests not run. Goals 7–20 Not started. Current candidates not approved for production.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update development roadmap with iPhone v3 research progress
</commit_message>
<xml_diff>
--- a/ProofCam_Android_Development_Roadmap.xlsx
+++ b/ProofCam_Android_Development_Roadmap.xlsx
@@ -9,10 +9,12 @@
   <sheets>
     <sheet name="20 Development Goals" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Scope and Decisions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Research Progress" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'20 Development Goals'!$A$1:$J$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'20 Development Goals'!$A$1:$M$21</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'20 Development Goals'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Research Progress'!$A$1:$D$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -44,8 +46,14 @@
       <name val="Calibri"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000563C1"/>
+      <sz val="11"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -55,6 +63,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="0017365D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF1F8"/>
       </patternFill>
     </fill>
   </fills>
@@ -70,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -79,6 +92,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -199,9 +221,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AndroidRoadmap" displayName="AndroidRoadmap" ref="A1:J21" headerRowCount="1">
-  <autoFilter ref="A1:J21"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="AndroidRoadmap" displayName="AndroidRoadmap" ref="A1:M21" headerRowCount="1">
+  <autoFilter ref="A1:M21"/>
+  <tableColumns count="13">
     <tableColumn id="1" name="Order"/>
     <tableColumn id="2" name="Phase"/>
     <tableColumn id="3" name="Goal"/>
@@ -212,6 +234,9 @@
     <tableColumn id="8" name="Suggested Owner"/>
     <tableColumn id="9" name="Technology / Spec"/>
     <tableColumn id="10" name="Status"/>
+    <tableColumn id="11" name="Progress as of 2026-09-27"/>
+    <tableColumn id="12" name="Remaining work / next action"/>
+    <tableColumn id="13" name="Evidence"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -506,7 +531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -519,6 +544,9 @@
     <col width="34" customWidth="1" min="8" max="8"/>
     <col width="55" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="65" customWidth="1" min="11" max="11"/>
+    <col width="65" customWidth="1" min="12" max="12"/>
+    <col width="43" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -572,6 +600,21 @@
           <t>Status</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Progress as of 2026-09-27</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Remaining work / next action</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="100" customHeight="1">
       <c r="A2" s="2" t="n">
@@ -622,6 +665,21 @@
           <t>Complete</t>
         </is>
       </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Product brief and pilot audience documented.</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Planning complete; implementation tracked below.</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>docs/01-product-brief.md</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="100" customHeight="1">
       <c r="A3" s="2" t="n">
@@ -649,7 +707,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Define Android support and reference tiers; assign accountability; use existing or freely borrowed devices and no paid services; defer iOS, video, editing, and browser UI.</t>
+          <t>Define Android support and reference tiers; assign accountability; use existing or freely borrowed devices and no paid services; defer production iOS, video, editing, and browser UI; permit the separate iPhone feasibility experiment.</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -670,6 +728,21 @@
       <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Complete</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Android pilot scope and free-only development constraints documented. iPhone research experiment subsequently authorized.</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Production iOS remains deferred; no paid services or hardware purchases.</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>docs/02-pilot-scope-and-free-development.md</t>
         </is>
       </c>
     </row>
@@ -722,6 +795,21 @@
           <t>Complete</t>
         </is>
       </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Threat model, privacy rules and assurance outcomes documented.</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Security controls still require implementation and validation.</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>docs/03-threat-model-and-privacy-policy.md</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="100" customHeight="1">
       <c r="A5" s="2" t="n">
@@ -772,6 +860,21 @@
           <t>Complete</t>
         </is>
       </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Capture/verification screens, states and clickable prototype delivered.</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Prototype behavior is simulated; production implementation pending.</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>docs/04-capture-and-verification-design.md</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="100" customHeight="1">
       <c r="A6" s="2" t="n">
@@ -822,8 +925,23 @@
           <t>In progress</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="100" customHeight="1">
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Harness, 11,200 distinct source images, 53 resolution variants and 300,000-case stress recipe plan prepared; tuning review recorded.</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Rights/content/near-duplicate review, final evaluation eligibility and real screenshots pending. Stress recipes are not completed evaluations.</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>docs/05-benchmark-data-and-harness.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="105" customHeight="1">
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
@@ -869,7 +987,22 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Blocked — device unavailable</t>
+          <t>Blocked</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Desktop study and Android research APK delivered. iPhone v3 default implemented: 125/125 marked simulations, 0/100 noise detections; all six previous v2 misses recovered. Linux regression and v3 AddressSanitizer checks pass.</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>No Android phone available. Run Mac validation, Apple codec tests and iPhone 16 Pro screenshot/performance/visual checks. V3 host median 4.392 s; no production qualification.</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>ios-benchmark/ADAPTIVE-V3.md</t>
         </is>
       </c>
     </row>
@@ -922,6 +1055,21 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>V3 selected only as iPhone research default; v1/v2 preserved. No production watermark or support envelope approved.</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Complete physical-device feasibility and quality gates before production selection.</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>ios-benchmark/TESTING.md</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="100" customHeight="1">
       <c r="A9" s="2" t="n">
@@ -972,6 +1120,21 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Repository and separate Android/iPhone research projects exist. Production Android foundation and CI goal not yet started.</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Proceed after goal 7; research APK/Xcode project does not satisfy production completion criteria.</t>
+        </is>
+      </c>
+      <c r="M9" s="4" t="inlineStr">
+        <is>
+          <t>README.md</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="100" customHeight="1">
       <c r="A10" s="2" t="n">
@@ -1022,6 +1185,17 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>No production implementation completed for this goal.</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Await listed prerequisites; research tests do not satisfy this release goal.</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr"/>
     </row>
     <row r="11" ht="100" customHeight="1">
       <c r="A11" s="2" t="n">
@@ -1072,6 +1246,17 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>No production implementation completed for this goal.</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Await listed prerequisites; research tests do not satisfy this release goal.</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr"/>
     </row>
     <row r="12" ht="100" customHeight="1">
       <c r="A12" s="2" t="n">
@@ -1122,6 +1307,17 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>No production implementation completed for this goal.</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Await listed prerequisites; research tests do not satisfy this release goal.</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr"/>
     </row>
     <row r="13" ht="100" customHeight="1">
       <c r="A13" s="2" t="n">
@@ -1172,6 +1368,17 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>No production implementation completed for this goal.</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Await listed prerequisites; research tests do not satisfy this release goal.</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr"/>
     </row>
     <row r="14" ht="100" customHeight="1">
       <c r="A14" s="2" t="n">
@@ -1222,6 +1429,17 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>No production implementation completed for this goal.</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Await listed prerequisites; research tests do not satisfy this release goal.</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr"/>
     </row>
     <row r="15" ht="100" customHeight="1">
       <c r="A15" s="2" t="n">
@@ -1272,6 +1490,17 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>No production implementation completed for this goal.</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Await listed prerequisites; research tests do not satisfy this release goal.</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr"/>
     </row>
     <row r="16" ht="100" customHeight="1">
       <c r="A16" s="2" t="n">
@@ -1322,6 +1551,17 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>No production implementation completed for this goal.</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Await listed prerequisites; research tests do not satisfy this release goal.</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr"/>
     </row>
     <row r="17" ht="100" customHeight="1">
       <c r="A17" s="2" t="n">
@@ -1372,6 +1612,17 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>No production implementation completed for this goal.</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Await listed prerequisites; research tests do not satisfy this release goal.</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr"/>
     </row>
     <row r="18" ht="100" customHeight="1">
       <c r="A18" s="2" t="n">
@@ -1422,6 +1673,17 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>No production implementation completed for this goal.</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Await listed prerequisites; research tests do not satisfy this release goal.</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr"/>
     </row>
     <row r="19" ht="100" customHeight="1">
       <c r="A19" s="2" t="n">
@@ -1472,6 +1734,17 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>No production implementation completed for this goal.</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Await listed prerequisites; research tests do not satisfy this release goal.</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr"/>
     </row>
     <row r="20" ht="100" customHeight="1">
       <c r="A20" s="2" t="n">
@@ -1522,6 +1795,17 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>No production implementation completed for this goal.</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Await listed prerequisites; research tests do not satisfy this release goal.</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr"/>
     </row>
     <row r="21" ht="100" customHeight="1">
       <c r="A21" s="2" t="n">
@@ -1572,9 +1856,20 @@
           <t>Not started</t>
         </is>
       </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>No production implementation completed for this goal.</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Await listed prerequisites; research tests do not satisfy this release goal.</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J21"/>
+  <autoFilter ref="A1:M21"/>
   <dataValidations count="1">
     <dataValidation sqref="J2:J21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Not started,In progress,Blocked,In review,Complete"</formula1>
@@ -1582,17 +1877,25 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId13"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId14"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1603,7 +1906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1622,7 +1925,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1">
+    <row r="2" ht="90" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Purpose</t>
@@ -1630,7 +1933,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>20 sequential development goals from incubation through deployment of the ProofCam Android photo pilot. This workbook is a proposed plan, not evidence of implemented capabilities.</t>
+          <t>20 development goals for the Android photo pilot, with progress recorded as of 2026-09-27. Research evidence does not imply production readiness.</t>
         </is>
       </c>
     </row>
@@ -1658,7 +1961,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="60" customHeight="1">
+    <row r="5" ht="90" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Deferred scope</t>
@@ -1666,11 +1969,11 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>iPhone, video/audio and partial-interval verification, browser verification UI, in-app editing, and stronger manufacturer sensor-origin assurance. These remain future work; this pilot does not fulfill the entire original first-release scope.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="60" customHeight="1">
+          <t>Production iPhone app, video/audio, partial-interval verification, browser verification, editing and manufacturer sensor-origin assurance remain deferred. A separate iPhone research app is now implemented for feasibility testing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="90" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Watermark choice</t>
@@ -1678,7 +1981,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Conventional watermarking first. Learned models are optional candidates only when benchmark evidence justifies them. Do not promise robustness before measurement.</t>
+          <t>Conventional watermarking first; no AI required for current research. iOS adaptive v3 is the research default, with v1/v2 selectable. Production selection awaits device, quality and support-envelope gates.</t>
         </is>
       </c>
     </row>
@@ -1754,7 +2057,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="60" customHeight="1">
+    <row r="13" ht="90" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Tracking</t>
@@ -1762,7 +2065,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Goals 1–4 planning/design complete. Goal 5 In progress (rights/final corpus/device evidence). Goal 6 desktop work complete; full goal Blocked — device unavailable, confirmed 2026-09-26. Research Android APK built; physical tests not run. Goals 7–20 Not started. Current candidates not approved for production.</t>
+          <t>Goals 1–4 complete as planning/design deliverables. Goal 5 in progress. Goal 6 host research implemented through iOS v3; Android device validation blocked and Mac/iPhone validation pending. Goals 7–20 remain not started as production goals; preparatory repository/research-app work is recorded separately.</t>
         </is>
       </c>
     </row>
@@ -1787,10 +2090,413 @@
       <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Existing or freely borrowed devices; local compute; free tools and licensed data; no paid services or store enrollment. Direct signed APK distribution. Public hosting/signing remains gated on compliant no-cost resources; never claim unavailable attestation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="75" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Available iPhone</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>User reports iPhone 16 Pro and current Xcode on their Mac. Mac validation and physical-device tests have not been run here. No Android phone is available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="75" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Latest implementation</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>dd40e45: adaptive iPhone v3, committed and pushed. Smaller repeated tiles, soft error correction, adaptive embedding and expanded geometric search.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="75" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Next action</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>On the Mac: pull latest code and run bash ios-benchmark/tools/validate-mac.sh. Then collect real iPhone screenshots, visual review and performance results. Android physical validation remains separately blocked.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="75" customWidth="1" min="2" max="2"/>
+    <col width="75" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Workstream / check</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Current result</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Status / limitation</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="75" customHeight="1">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Snapshot</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Updated 2026-09-27; implementation dd40e45.</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Free-only development. Research app, not production release.</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="75" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>iPhone app</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>SwiftUI/Xcode project prepared; adaptive v3 default; v1/v2 selectable.</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Apple SDK build, signing, simulator and device execution pending.</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>ios-benchmark/README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="75" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>V3 geometric simulation</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>125/125 marked cases recovered: 25 transforms on five sources. Includes resizes, crops, rotations, mirrors, JPEG and synthetic viewer chrome.</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Three development sources plus two preselected additional photos; not broad release qualification.</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>benchmark/reports/step06-ios-adaptive-simulation.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="75" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Previous failures</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Original three sources: v2 69/75 → v3 75/75. Two additional photos: 50/50.</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>All six previous v2 misses fixed in this simulation; arbitrary combinations not guaranteed.</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>benchmark/reports/step06-ios-adaptive-comparison.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="75" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Negative simulation</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>No detections on 100 unmarked procedural noise inputs; no unexpected IDs in all 225 cases.</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Not a natural-photo false-positive study or cryptographic validation.</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>benchmark/reports/step06-ios-adaptive-simulation.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="75" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Linux Release regression</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>34 discovered: 30 passed, four optional tests skipped; zero failures. Simulation executed separately.</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Skipped: two fixture generators, optional diagnostic, separately run simulation.</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>benchmark/reports/step06-ios-adaptive-validation.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="75" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>AddressSanitizer</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Five active v3 tests passed; two optional tests skipped; no errors.</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>Leak detection disabled; not full simulation or Apple code coverage.</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>benchmark/reports/step06-ios-adaptive-validation.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="75" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Project checks</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>App Swift syntax parse and deterministic Xcode project generation passed.</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Not Apple SDK typechecking or Xcode build evidence.</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>benchmark/reports/step06-ios-adaptive-validation.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="75" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>Image quality</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Photo SSIM v2→v3: 0.941→0.958; 0.912→0.950; 0.947→0.962.</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>PSNR not uniformly improved; procedural noise quality worsened. Invisibility and Apple JPEG quality not qualified.</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>benchmark/reports/step06-ios-adaptive-comparison.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="75" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Host recovery time</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Median 4.392 s; p95 6.903 s; maximum 8.953 s across 225 cases.</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Slower than v2; not iPhone timing or a mobile latency pass.</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>benchmark/reports/step06-ios-adaptive-comparison.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="75" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Apple codec checks</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Six Apple-only tests prepared.</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Not executed; run Mac validation script.</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>ios-benchmark/tools/validate-mac.sh</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="75" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Physical iPhone evidence</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>iPhone 16 Pro available to user.</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Pending Mac build and actual screenshots, display review, latency and memory measurements.</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>ios-benchmark/TESTING.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="75" customHeight="1">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>Physical Android evidence</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Research APK built; no Android phone available.</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Blocked; iOS results do not qualify Android.</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>docs/06-conventional-watermark-final-report.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="75" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Production gate</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>No production candidate selected; deployment not started.</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Goals 5/6 remain incomplete; goals 7–20 remain open.</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>docs/06-conventional-watermark-final-report.md</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D15"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId14"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Build local signed provenance service and iPhone capture request flow
</commit_message>
<xml_diff>
--- a/ProofCam_Android_Development_Roadmap.xlsx
+++ b/ProofCam_Android_Development_Roadmap.xlsx
@@ -10,11 +10,13 @@
     <sheet name="20 Development Goals" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Scope and Decisions" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Research Progress" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Provenance Progress" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'20 Development Goals'!$A$1:$M$21</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'20 Development Goals'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Research Progress'!$A$1:$D$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Provenance Progress'!$A$1:$D$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1136,7 +1138,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="100" customHeight="1">
+    <row r="10" ht="105" customHeight="1">
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
@@ -1182,22 +1184,26 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>No production implementation completed for this goal.</t>
+          <t>Development protocol implemented: deterministic CBOR, COSE_Sign1 ES256, typed requests, SHA-256 exact-file certificates, trust expiry/status, replay/idempotency rules and cross-language vectors.</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Await listed prerequisites; research tests do not satisfy this release goal.</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11" ht="100" customHeight="1">
+          <t>Production schema review, canonical-pixel integrity, Rust integration, production trust lifecycle and independent review remain pending.</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>provenance/PROTOCOL.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="105" customHeight="1">
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
@@ -1248,17 +1254,21 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>No production implementation completed for this goal.</t>
+          <t>Android production capture not started. Separate iPhone camera-only research path now prepares finalized watermarked JPEGs and signed requests.</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Await listed prerequisites; research tests do not satisfy this release goal.</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr"/>
-    </row>
-    <row r="12" ht="100" customHeight="1">
+          <t>Mac build and physical iPhone camera validation pending; Android CameraX implementation and reference-device checks still pending.</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>ios-benchmark/ProofCamResearch/CaptureProvenance.swift</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="105" customHeight="1">
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
@@ -1309,17 +1319,21 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>No production implementation completed for this goal.</t>
+          <t>Android production pipeline not started. iPhone research capture embeds v3, writes/reopens the final JPEG, hashes its exact bytes and signs an offline request.</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Await listed prerequisites; research tests do not satisfy this release goal.</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr"/>
-    </row>
-    <row r="13" ht="100" customHeight="1">
+          <t>Production watermark selection, canonical integrity, Android/Rust bindings and phone quality/performance gates remain open.</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>provenance/README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="105" customHeight="1">
       <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
@@ -1365,22 +1379,26 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>No production implementation completed for this goal.</t>
+          <t>Development enrollment admits invited P-256 keys after proof of possession; backend issues bound one-use challenges. iPhone Secure Enclave signing path prepared.</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>Await listed prerequisites; research tests do not satisfy this release goal.</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="inlineStr"/>
-    </row>
-    <row r="14" ht="100" customHeight="1">
+          <t>No server platform-attestation validator. Hardware/app/camera assurance remains unavailable. Android Keystore integration and real-device testing pending.</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>provenance/README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="105" customHeight="1">
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
@@ -1426,22 +1444,26 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>No production implementation completed for this goal.</t>
+          <t>Local Python/SQLite development service implements atomic challenge consumption, signed certificate issuance, durable request idempotency, conflicts and per-installation quotas.</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>Await listed prerequisites; research tests do not satisfy this release goal.</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15" ht="100" customHeight="1">
+          <t>Protected production signer, Rust/PostgreSQL deployment, TLS/operations and attestation gates pending. Development issuers rejected by default.</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>provenance/service.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="105" customHeight="1">
       <c r="A15" s="2" t="n">
         <v>14</v>
       </c>
@@ -1492,17 +1514,21 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>No production implementation completed for this goal.</t>
+          <t>Production Android queue/sharing not started. iPhone stores pending JPEG/request pairs; Mac CLI submits persisted requests with idempotent manual retries.</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>Await listed prerequisites; research tests do not satisfy this release goal.</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="inlineStr"/>
-    </row>
-    <row r="16" ht="100" customHeight="1">
+          <t>Automatic mobile synchronization/reconciliation, complete interruption testing and production share-state flow remain pending.</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>provenance/README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="105" customHeight="1">
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
@@ -1548,22 +1574,26 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>No production implementation completed for this goal.</t>
+          <t>Independent local verifier checks issuer signatures/trust and exact file hashes; rejects changed files, wrong IDs and development issuers unless explicitly enabled.</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Await listed prerequisites; research tests do not satisfy this release goal.</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr"/>
-    </row>
-    <row r="17" ht="100" customHeight="1">
+          <t>Android UI/integration, canonical-pixel comparison and production trust remain pending. Verification does not establish camera origin or absence of AI.</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>provenance/verifier.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="105" customHeight="1">
       <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
@@ -1609,20 +1639,24 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>No production implementation completed for this goal.</t>
+          <t>Development backend supports fresh owner-signed removal, installation revocation and ID-only non-reuse tombstones.</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>Await listed prerequisites; research tests do not satisfy this release goal.</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr"/>
+          <t>Recovery credentials, app management UI, authoritative deletion journal/restore reconciliation and policy retention jobs remain pending.</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>provenance/service.py</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="100" customHeight="1">
       <c r="A18" s="2" t="n">
@@ -1889,13 +1923,21 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId21"/>
   </hyperlinks>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId14"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId22"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1906,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2057,7 +2099,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="90" customHeight="1">
+    <row r="13" ht="110" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Tracking</t>
@@ -2065,7 +2107,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Goals 1–4 complete as planning/design deliverables. Goal 5 in progress. Goal 6 host research implemented through iOS v3; Android device validation blocked and Mac/iPhone validation pending. Goals 7–20 remain not started as production goals; preparatory repository/research-app work is recorded separately.</t>
+          <t>Goals 1–4 planning/design complete; goal 5 in progress; goal 6 blocked on Android hardware and pending Mac/iPhone validation. Goals 9, 12, 13, 15 and 16 now in progress through development provenance infrastructure; no production gate is complete. Other implementation/release goals remain not started, with research precursors noted.</t>
         </is>
       </c>
     </row>
@@ -2113,7 +2155,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>dd40e45: adaptive iPhone v3, committed and pushed. Smaller repeated tiles, soft error correction, adaptive embedding and expanded geometric search.</t>
+          <t>Adaptive iPhone v3 is preserved. Local provenance service, independent verifier, protocol tests and iPhone camera/Secure Enclave request-export path now implemented; native Apple execution remains pending.</t>
         </is>
       </c>
     </row>
@@ -2125,7 +2167,19 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>On the Mac: pull latest code and run bash ios-benchmark/tools/validate-mac.sh. Then collect real iPhone screenshots, visual review and performance results. Android physical validation remains separately blocked.</t>
+          <t>On Mac: run ios-benchmark/tools/validate-mac.sh, install on iPhone, test camera/enrollment/Secure Enclave and exported-file verification via the local provenance service. Production attestation and signing remain open. Android hardware is still unavailable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="95" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Provenance trust boundary</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>All certificates are development records. Exact-byte match is supported; server-attested camera origin and absence of AI are not established. Local Python/SQLite is a reference implementation, not production Rust/PostgreSQL deployment.</t>
         </is>
       </c>
     </row>
@@ -2179,7 +2233,7 @@
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Updated 2026-09-27; implementation dd40e45.</t>
+          <t>Watermark snapshot: v3 implementation dd40e45. See Provenance Progress for the new infrastructure.</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
@@ -2499,4 +2553,187 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="75" customWidth="1" min="2" max="2"/>
+    <col width="75" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Implemented progress</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Remaining validation / limits</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="90" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Enrollment and keys</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Private invitation admission, P-256 proof of possession, server-side revocation; native Secure Enclave signing code.</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Native key protection not server-attested; Apple execution pending.</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>provenance/README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="90" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Registration service</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Bound challenges, atomic record creation, exact retry after restart, conflict rejection, quotas and no media upload.</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Local development only; no production protected signer, attestation validator or public deployment.</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>provenance/service.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="90" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Independent verification</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>COSE signatures, trusted issuer status/expiry, expected-ID check and exact-file SHA-256 comparison.</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Development opt-in required. Camera origin and absence of AI never reported verified.</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>provenance/verifier.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="90" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Camera capture and export</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Camera-only route; v3 watermark; final JPEG stored/reopened/hashed; signed offline request; pending files retained across launches.</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Mac build and device tests pending. Manual transfer/submission; no automatic mobile registration.</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>ios-benchmark/ProofCamResearch/CaptureProvenance.swift</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="90" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Protocol and tests</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>22 backend security/integration tests pass, including real HTTP and separate-process CLI; four Swift/Python byte-vector tests prepared and run in the portable suite.</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Apple CryptoKit tests and physical camera/storage/keychain tests remain pending; no independent security audit.</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>provenance/validation.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="90" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Removal and revocation</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Owner signature and fresh management challenge; atomic removal/non-reuse tombstone; installation revocation.</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Accountless recovery, retention automation and authoritative restore journal pending.</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>provenance/PROTOCOL.md</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D7"/>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Harden provenance file I/O and expand adversarial validation
</commit_message>
<xml_diff>
--- a/ProofCam_Android_Development_Roadmap.xlsx
+++ b/ProofCam_Android_Development_Roadmap.xlsx
@@ -1449,7 +1449,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Local Python/SQLite development service implements atomic challenge consumption, signed certificate issuance, durable request idempotency, conflicts and per-installation quotas.</t>
+          <t>Local development registration service and independent verifier implemented. Follow-up audit: 37 backend tests pass; abrupt process exits, races, malformed requests and OpenSSL signatures checked. Atomic export and special-file input defects fixed.</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -2147,7 +2147,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="75" customHeight="1">
+    <row r="17" ht="100" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Latest implementation</t>
@@ -2155,7 +2155,7 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Adaptive iPhone v3 is preserved. Local provenance service, independent verifier, protocol tests and iPhone camera/Secure Enclave request-export path now implemented; native Apple execution remains pending.</t>
+          <t>Local signed provenance infrastructure plus iPhone camera/Secure Enclave export path prepared. Follow-up audit fixed atomic local-file publication and rejection of blocking special-file inputs. 37 backend tests pass; Apple/device validation is still pending.</t>
         </is>
       </c>
     </row>
@@ -2680,7 +2680,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="90" customHeight="1">
+    <row r="6" ht="115" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Protocol and tests</t>
@@ -2688,12 +2688,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>22 backend security/integration tests pass, including real HTTP and separate-process CLI; four Swift/Python byte-vector tests prepared and run in the portable suite.</t>
+          <t>37 backend tests pass: crash/restart, concurrent ownership/enrollment, OpenSSL interoperability, 3,296 single-bit request mutations, 2,000 seeded malformed messages and file/HTTP bounds. Swift: 34 pass, four optional skips.</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Apple CryptoKit tests and physical camera/storage/keychain tests remain pending; no independent security audit.</t>
+          <t>Two defects fixed: partial file publication after failed save and blocking special-file reads. Four pinned Python packages returned no OSV advisories at check time. Apple/device tests and independent security audit remain pending.</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Add opt-in App Attest validation and iPhone evidence handoff
</commit_message>
<xml_diff>
--- a/ProofCam_Android_Development_Roadmap.xlsx
+++ b/ProofCam_Android_Development_Roadmap.xlsx
@@ -604,7 +604,7 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Progress as of 2026-09-27</t>
+          <t>Progress as of 2026-09-28</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -1384,17 +1384,17 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Development enrollment admits invited P-256 keys after proof of possession; backend issues bound one-use challenges. iPhone Secure Enclave signing path prepared.</t>
+          <t>Development signing, verification and optional server App Attest cryptographic checks implemented; native challenge/export flow prepared.</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>No server platform-attestation validator. Hardware/app/camera assurance remains unavailable. Android Keystore integration and real-device testing pending.</t>
+          <t>Live Apple evidence and eligible provisioning, receipt risk/revocation checks, Android attestation, production issuer and device qualification pending. Free Personal Team cannot enable App Attest.</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>provenance/README.md</t>
+          <t>provenance/APP-ATTEST.md; provenance/validation.json</t>
         </is>
       </c>
     </row>
@@ -1948,7 +1948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2180,6 +2180,18 @@
       <c r="B19" s="3" t="inlineStr">
         <is>
           <t>All certificates are development records. Exact-byte match is supported; server-attested camera origin and absence of AI are not established. Local Python/SQLite is a reference implementation, not production Rust/PostgreSQL deployment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>App Attest activation</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>No purchases. Optional implementation remains OFF unless an existing eligible Apple team/profile is available. Free Personal Team lacks this capability; live verification pending.</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2688,12 +2700,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>37 backend tests pass: crash/restart, concurrent ownership/enrollment, OpenSSL interoperability, 3,296 single-bit request mutations, 2,000 seeded malformed messages and file/HTTP bounds. Swift: 34 pass, four optional skips.</t>
+          <t>52 backend tests pass, including 15 synthetic App Attest tests; 3,296 bit mutations and 2,000 malformed messages rejected. Swift: 37 pass, four optional skips. App syntax and deterministic project generation pass.</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Two defects fixed: partial file publication after failed save and blocking special-file reads. Four pinned Python packages returned no OSV advisories at check time. Apple/device tests and independent security audit remain pending.</t>
+          <t>Synthetic attestation positives only; no genuine Apple acceptance, Apple SDK build or physical-device tests. Independent security audit pending.</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -2721,6 +2733,28 @@
       <c r="D7" s="4" t="inlineStr">
         <is>
           <t>provenance/PROTOCOL.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="100" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>App Attest cryptographic layer</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Pinned Apple root; app/environment/build policy; fresh challenge; request-bound assertion; monotonic counter; atomic replay/downgrade protection; saved exact retries. Native integration defaults OFF.</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Requires existing eligible Apple team/profile; free Personal Team unsupported. Receipt risk/revocation and live Apple checks pending. Does not prove camera origin or absence of AI.</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>provenance/APP-ATTEST.md; provenance/validation.json</t>
         </is>
       </c>
     </row>

</xml_diff>